<commit_message>
ajustes de comportamiento y ajuste conforme a documentacion
</commit_message>
<xml_diff>
--- a/docs/CHECKLIST_PENDIENTES.xlsx
+++ b/docs/CHECKLIST_PENDIENTES.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="411">
   <si>
     <t>NeoEduCore — Avance de pendientes</t>
   </si>
@@ -160,7 +160,7 @@
     <t>D3</t>
   </si>
   <si>
-    <t>Expiración de sesión: 60 min (informe) vs. 12 h (sistema)</t>
+    <t>Expiracion de sesion: inactividad de 60 min</t>
   </si>
   <si>
     <t>• config/sanctum.php:50 → SANCTUM_TOKEN_EXPIRATION_MINUTES, 720 por defecto.
@@ -171,6 +171,9 @@
     <t>ESTADO_Y_PENDIENTES.md §9.3 · ANALISIS_MODELO_DATOS_TFG.md §10.2 nº 9</t>
   </si>
   <si>
+    <t>Inactividad real de 60 min sobre last_used_at (SANCTUM_TOKEN_INACTIVITY_MINUTES), no expiracion absoluta. Bajar EXPIRATION a 60 habria expulsado al alumno a mitad de un examen de hasta 300 min. Via Sanctum::authenticateAccessTokensUsing(), no middleware. Cierra K9 e I-11.</t>
+  </si>
+  <si>
     <t>D4</t>
   </si>
   <si>
@@ -181,6 +184,9 @@
   </si>
   <si>
     <t>ESTADO_Y_PENDIENTES.md §3.6 nº 8</t>
+  </si>
+  <si>
+    <t>Campo ai_notice en la respuesta del chat y del diagnostico. Texto en openai.tutor.notice (OPENAI_TUTOR_NOTICE). Se eligio el sistema y no el frontend: el compromiso de [397] es del sistema. Cierra K5.</t>
   </si>
   <si>
     <t>D5</t>
@@ -196,6 +202,9 @@
     <t>ESTADO_Y_PENDIENTES.md §9.3 · §3.6 nº 6</t>
   </si>
   <si>
+    <t>Tabla ai_tutor_incidents (migracion 2026_09_13_000003, aplicada) + GET /platform/ai-tutor-metrics solo superadmin, solo agregados. NO guarda el texto que provoco la incidencia. Cierra K6.</t>
+  </si>
+  <si>
     <t>D6</t>
   </si>
   <si>
@@ -208,6 +217,9 @@
     <t>ESTADO_Y_PENDIENTES.md §8</t>
   </si>
   <si>
+    <t>Se queda sin activar (la regla no se toca) pero la respuesta devuelve status, can_sign_in y activation_needed, y el mensaje dice que hay que enviar el enlace de activacion.</t>
+  </si>
+  <si>
     <t>D7</t>
   </si>
   <si>
@@ -217,6 +229,9 @@
     <t>• Se dejó para poder mostrar «intento 2 de 3». Confirmar.</t>
   </si>
   <si>
+    <t>Confirmado: se queda. Sin cambios de codigo. Con max_attempts y submitted_count el frontend pinta «intento 2 de 3». No es informacion sensible.</t>
+  </si>
+  <si>
     <t>D8</t>
   </si>
   <si>
@@ -227,6 +242,9 @@
   </si>
   <si>
     <t>ESTADO_Y_PENDIENTES.md §5, pendientes 31/07</t>
+  </si>
+  <si>
+    <t>Migracion 2026_09_13_000004 sobre 26 tablas, idempotente, aplicada. RLS sin politicas no afecta a la app (su rol es propietario); cierra la API REST automatica de Supabase. Ademas schema:dump-sql ya no pierde el bloque.</t>
   </si>
   <si>
     <t>S1</t>
@@ -367,7 +385,11 @@
     <t>P2.7</t>
   </si>
   <si>
-    <t>SANCTUM_TOKEN_EXPIRATION_MINUTES según D3</t>
+    <t>SANCTUM_TOKEN_EXPIRATION_MINUTES=720 y SANCTUM_TOKEN_INACTIVITY_MINUTES=60</t>
+  </si>
+  <si>
+    <t>• Las dos, segun D3.
+• EXPIRATION es el tope absoluto de jornada; INACTIVITY es lo que exige [758].</t>
   </si>
   <si>
     <t>P3</t>
@@ -540,6 +562,9 @@
     <t>• (según D4)</t>
   </si>
   <si>
+    <t>Listo para consumir: el backend lo manda en data.ai_notice (D4).</t>
+  </si>
+  <si>
     <t>F8</t>
   </si>
   <si>
@@ -765,6 +790,9 @@
     <t>• según D3</t>
   </si>
   <si>
+    <t>Se cumple [758] desde D3. Explicar que es inactividad y no expiracion absoluta, y por que.</t>
+  </si>
+  <si>
     <t>C1</t>
   </si>
   <si>
@@ -816,6 +844,9 @@
     <t>Criterio 75 % automático [173] vs. revisión humana [396]</t>
   </si>
   <si>
+    <t>El 75 % ya es medible (D5); queda decidir que dice el informe sobre la revision humana.</t>
+  </si>
+  <si>
     <t>K1</t>
   </si>
   <si>
@@ -861,12 +892,18 @@
     <t>Aviso de IA en cada intervención [397] → según D4</t>
   </si>
   <si>
+    <t>El sistema envia el aviso en ai_notice (D4).</t>
+  </si>
+  <si>
     <t>K6</t>
   </si>
   <si>
     <t>«Registrará incidencias» / 75 % [173] → según D5</t>
   </si>
   <si>
+    <t>Hay tabla de incidencias y el 75 % se calcula (D5).</t>
+  </si>
+  <si>
     <t>K7</t>
   </si>
   <si>
@@ -883,6 +920,9 @@
   </si>
   <si>
     <t>Sesión de 60 min [758] → según D3</t>
+  </si>
+  <si>
+    <t>El sistema caduca por inactividad a los 60 min (D3).</t>
   </si>
   <si>
     <t>K10</t>
@@ -1230,6 +1270,20 @@
   </si>
   <si>
     <t>ESTADO_Y_PENDIENTES.md, pendientes 13/09/2026</t>
+  </si>
+  <si>
+    <t>F17</t>
+  </si>
+  <si>
+    <t>Panel de metricas del tutor IA para el superadmin</t>
+  </si>
+  <si>
+    <t>• Datos: GET /platform/ai-tutor-metrics (ventana, totales, validation_pass_rate, por tipo, por etapa, por institucion y serie diaria).
+• El umbral de [173] es 75 %: conviene que se vea si se cumple o no de un vistazo.
+• Solo agregados: no hay ningun dato de alumno que mostrar.</t>
+  </si>
+  <si>
+    <t>ESTADO_Y_PENDIENTES.md, seccion Aviso de IA e incidencias</t>
   </si>
 </sst>
 </file>
@@ -1804,7 +1858,7 @@
       </c>
       <c r="C5">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A5,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D5">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A5,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -1812,7 +1866,7 @@
       </c>
       <c r="E5">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A5,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F5">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A5,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
@@ -1820,11 +1874,11 @@
       </c>
       <c r="G5">
         <f>E5+F5</f>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H5" s="16">
         <f>IF(B5=0,0,G5/B5)</f>
-        <v>0.22222222222222</v>
+        <v>0.88888888888889</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1932,11 +1986,11 @@
       </c>
       <c r="B9">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A9,Checklist!$B$2:$B$327,"Tarea")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A9,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A9,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -1969,7 +2023,7 @@
       </c>
       <c r="C10">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A10,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D10">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A10,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -1981,15 +2035,15 @@
       </c>
       <c r="F10">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A10,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G10">
         <f>E10+F10</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H10" s="16">
         <f>IF(B10=0,0,G10/B10)</f>
-        <v>0.097560975609756</v>
+        <v>0.17073170731707</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2097,11 +2151,11 @@
       </c>
       <c r="B14" s="15">
         <f>SUM(B5:B13)</f>
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" s="15">
         <f>SUM(C5:C13)</f>
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D14" s="15">
         <f>SUM(D5:D13)</f>
@@ -2109,19 +2163,19 @@
       </c>
       <c r="E14" s="15">
         <f>SUM(E5:E13)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F14" s="15">
         <f>SUM(F5:F13)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G14" s="15">
         <f>SUM(G5:G13)</f>
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H14" s="17">
         <f>IF(B14=0,0,G14/B14)</f>
-        <v>0.077669902912621</v>
+        <v>0.16346153846154</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -2160,7 +2214,7 @@
       </c>
       <c r="C17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -2168,7 +2222,7 @@
       </c>
       <c r="E17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
@@ -2176,11 +2230,11 @@
       </c>
       <c r="G17">
         <f>E17+F17</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" s="16">
         <f>IF(B17=0,0,G17/B17)</f>
-        <v>0.083333333333333</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -2189,11 +2243,11 @@
       </c>
       <c r="B18">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A18,Checklist!$B$2:$B$327,"Tarea")</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C18">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A18,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D18">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A18,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -2213,7 +2267,7 @@
       </c>
       <c r="H18" s="16">
         <f>IF(B18=0,0,G18/B18)</f>
-        <v>0.14285714285714</v>
+        <v>0.13333333333333</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2226,7 +2280,7 @@
       </c>
       <c r="C19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -2234,7 +2288,7 @@
       </c>
       <c r="E19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
@@ -2242,11 +2296,11 @@
       </c>
       <c r="G19">
         <f>E19+F19</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H19" s="16">
         <f>IF(B19=0,0,G19/B19)</f>
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -2259,7 +2313,7 @@
       </c>
       <c r="C20">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A20,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D20">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A20,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -2267,19 +2321,19 @@
       </c>
       <c r="E20">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A20,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F20">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A20,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G20">
         <f>E20+F20</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H20" s="16">
         <f>IF(B20=0,0,G20/B20)</f>
-        <v>0.066666666666667</v>
+        <v>0.16666666666667</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -2288,11 +2342,11 @@
       </c>
       <c r="B21" s="15">
         <f>SUM(B17:B20)</f>
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C21" s="15">
         <f>SUM(C17:C20)</f>
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D21" s="15">
         <f>SUM(D17:D20)</f>
@@ -2300,19 +2354,19 @@
       </c>
       <c r="E21" s="15">
         <f>SUM(E17:E20)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F21" s="15">
         <f>SUM(F17:F20)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G21" s="15">
         <f>SUM(G17:G20)</f>
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H21" s="17">
         <f>IF(B21=0,0,G21/B21)</f>
-        <v>0.077669902912621</v>
+        <v>0.16346153846154</v>
       </c>
     </row>
   </sheetData>
@@ -2496,14 +2550,18 @@
         <v>47</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K4" s="8"/>
-      <c r="L4" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="K4" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>27</v>
@@ -2516,24 +2574,28 @@
         <v>22</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5" s="8"/>
-      <c r="L5" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="K5" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>27</v>
@@ -2546,24 +2608,28 @@
         <v>22</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K6" s="8"/>
-      <c r="L6" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="K6" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>27</v>
@@ -2576,24 +2642,28 @@
         <v>23</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K7" s="8"/>
-      <c r="L7" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="K7" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>27</v>
@@ -2606,22 +2676,26 @@
         <v>23</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K8" s="8"/>
-      <c r="L8" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="K8" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>27</v>
@@ -2634,24 +2708,28 @@
         <v>23</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K9" s="8"/>
-      <c r="L9" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="K9" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>27</v>
@@ -2664,10 +2742,10 @@
         <v>20</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -2679,7 +2757,7 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>27</v>
@@ -2692,10 +2770,10 @@
         <v>20</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -2707,7 +2785,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>27</v>
@@ -2720,7 +2798,7 @@
         <v>20</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -2733,10 +2811,10 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="3" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>11</v>
@@ -2746,7 +2824,7 @@
         <v>20</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -2759,10 +2837,10 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>11</v>
@@ -2772,7 +2850,7 @@
         <v>20</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
@@ -2785,7 +2863,7 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>27</v>
@@ -2798,10 +2876,10 @@
         <v>21</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -2812,12 +2890,12 @@
         <v>46278.0</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>27</v>
@@ -2830,14 +2908,14 @@
         <v>20</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>4</v>
@@ -2847,10 +2925,10 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="3" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>12</v>
@@ -2860,7 +2938,7 @@
         <v>20</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -2873,10 +2951,10 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>12</v>
@@ -2886,10 +2964,10 @@
         <v>20</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -2901,10 +2979,10 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>12</v>
@@ -2914,7 +2992,7 @@
         <v>20</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
@@ -2927,7 +3005,7 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>27</v>
@@ -2940,10 +3018,10 @@
         <v>20</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -2955,10 +3033,10 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="3" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>12</v>
@@ -2968,7 +3046,7 @@
         <v>20</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
@@ -2981,10 +3059,10 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>12</v>
@@ -2994,7 +3072,7 @@
         <v>20</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
@@ -3007,10 +3085,10 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>12</v>
@@ -3020,7 +3098,7 @@
         <v>20</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
@@ -3033,10 +3111,10 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>12</v>
@@ -3046,7 +3124,7 @@
         <v>20</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
@@ -3059,10 +3137,10 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>12</v>
@@ -3072,7 +3150,7 @@
         <v>20</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
@@ -3085,10 +3163,10 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>12</v>
@@ -3098,7 +3176,7 @@
         <v>20</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
@@ -3111,10 +3189,10 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>12</v>
@@ -3124,9 +3202,11 @@
         <v>20</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="G27" s="3"/>
+        <v>117</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>118</v>
+      </c>
       <c r="H27" s="3" t="s">
         <v>44</v>
       </c>
@@ -3139,7 +3219,7 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="2" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>27</v>
@@ -3152,10 +3232,10 @@
         <v>20</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -3167,7 +3247,7 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" s="2" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>27</v>
@@ -3180,14 +3260,14 @@
         <v>21</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="H29" s="2"/>
       <c r="I29" s="2" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>4</v>
@@ -3197,7 +3277,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" s="2" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>27</v>
@@ -3210,10 +3290,10 @@
         <v>23</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
@@ -3225,7 +3305,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="2" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>27</v>
@@ -3238,10 +3318,10 @@
         <v>21</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -3253,7 +3333,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="2" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>27</v>
@@ -3266,10 +3346,10 @@
         <v>21</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -3281,7 +3361,7 @@
     </row>
     <row r="33" spans="1:12">
       <c r="A33" s="2" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>27</v>
@@ -3294,10 +3374,10 @@
         <v>23</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -3309,7 +3389,7 @@
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>27</v>
@@ -3322,13 +3402,13 @@
         <v>20</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2" t="s">
@@ -3339,7 +3419,7 @@
     </row>
     <row r="35" spans="1:12">
       <c r="A35" s="2" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>27</v>
@@ -3352,16 +3432,16 @@
         <v>23</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>4</v>
@@ -3371,7 +3451,7 @@
     </row>
     <row r="36" spans="1:12">
       <c r="A36" s="2" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>27</v>
@@ -3384,13 +3464,13 @@
         <v>23</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="G36" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="H36" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2" t="s">
@@ -3401,7 +3481,7 @@
     </row>
     <row r="37" spans="1:12">
       <c r="A37" s="2" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>27</v>
@@ -3414,10 +3494,10 @@
         <v>21</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -3429,7 +3509,7 @@
     </row>
     <row r="38" spans="1:12">
       <c r="A38" s="2" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>27</v>
@@ -3438,16 +3518,16 @@
         <v>14</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -3459,7 +3539,7 @@
     </row>
     <row r="39" spans="1:12">
       <c r="A39" s="2" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>27</v>
@@ -3468,16 +3548,16 @@
         <v>14</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
@@ -3489,7 +3569,7 @@
     </row>
     <row r="40" spans="1:12">
       <c r="A40" s="2" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>27</v>
@@ -3498,16 +3578,16 @@
         <v>14</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -3519,7 +3599,7 @@
     </row>
     <row r="41" spans="1:12">
       <c r="A41" s="2" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>27</v>
@@ -3528,16 +3608,16 @@
         <v>14</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
@@ -3549,7 +3629,7 @@
     </row>
     <row r="42" spans="1:12">
       <c r="A42" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>27</v>
@@ -3558,16 +3638,16 @@
         <v>14</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
@@ -3579,7 +3659,7 @@
     </row>
     <row r="43" spans="1:12">
       <c r="A43" s="2" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>27</v>
@@ -3588,16 +3668,16 @@
         <v>14</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -3609,7 +3689,7 @@
     </row>
     <row r="44" spans="1:12">
       <c r="A44" s="2" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>27</v>
@@ -3618,30 +3698,32 @@
         <v>14</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2" t="s">
         <v>4</v>
       </c>
       <c r="K44" s="8"/>
-      <c r="L44" s="2"/>
+      <c r="L44" s="2" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="45" spans="1:12">
       <c r="A45" s="2" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>27</v>
@@ -3650,16 +3732,16 @@
         <v>14</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
@@ -3671,7 +3753,7 @@
     </row>
     <row r="46" spans="1:12">
       <c r="A46" s="2" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>27</v>
@@ -3680,13 +3762,13 @@
         <v>14</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
@@ -3699,7 +3781,7 @@
     </row>
     <row r="47" spans="1:12">
       <c r="A47" s="2" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>27</v>
@@ -3708,16 +3790,16 @@
         <v>14</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
@@ -3729,7 +3811,7 @@
     </row>
     <row r="48" spans="1:12">
       <c r="A48" s="2" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>27</v>
@@ -3738,16 +3820,16 @@
         <v>14</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
@@ -3759,7 +3841,7 @@
     </row>
     <row r="49" spans="1:12">
       <c r="A49" s="2" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>27</v>
@@ -3768,13 +3850,13 @@
         <v>14</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
@@ -3787,22 +3869,22 @@
     </row>
     <row r="50" spans="1:12">
       <c r="A50" s="3" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
@@ -3815,22 +3897,22 @@
     </row>
     <row r="51" spans="1:12">
       <c r="A51" s="3" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="3"/>
@@ -3843,22 +3925,22 @@
     </row>
     <row r="52" spans="1:12">
       <c r="A52" s="3" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
@@ -3871,7 +3953,7 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53" s="2" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>27</v>
@@ -3880,16 +3962,16 @@
         <v>14</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
@@ -3901,7 +3983,7 @@
     </row>
     <row r="54" spans="1:12">
       <c r="A54" s="2" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>27</v>
@@ -3910,16 +3992,16 @@
         <v>14</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
@@ -3931,7 +4013,7 @@
     </row>
     <row r="55" spans="1:12">
       <c r="A55" s="2" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>27</v>
@@ -3940,16 +4022,16 @@
         <v>14</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
@@ -3961,7 +4043,7 @@
     </row>
     <row r="56" spans="1:12">
       <c r="A56" s="2" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>27</v>
@@ -3970,13 +4052,13 @@
         <v>14</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
@@ -3989,7 +4071,7 @@
     </row>
     <row r="57" spans="1:12">
       <c r="A57" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>27</v>
@@ -3998,16 +4080,16 @@
         <v>15</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
@@ -4019,22 +4101,22 @@
     </row>
     <row r="58" spans="1:12">
       <c r="A58" s="3" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
@@ -4047,22 +4129,22 @@
     </row>
     <row r="59" spans="1:12">
       <c r="A59" s="3" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
@@ -4075,22 +4157,22 @@
     </row>
     <row r="60" spans="1:12">
       <c r="A60" s="3" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
@@ -4103,22 +4185,22 @@
     </row>
     <row r="61" spans="1:12">
       <c r="A61" s="3" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
@@ -4131,7 +4213,7 @@
     </row>
     <row r="62" spans="1:12">
       <c r="A62" s="2" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>27</v>
@@ -4140,16 +4222,16 @@
         <v>15</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
@@ -4161,7 +4243,7 @@
     </row>
     <row r="63" spans="1:12">
       <c r="A63" s="2" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>27</v>
@@ -4170,16 +4252,16 @@
         <v>15</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>34</v>
@@ -4190,12 +4272,12 @@
       </c>
       <c r="K63" s="8"/>
       <c r="L63" s="2" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="64" spans="1:12">
       <c r="A64" s="2" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>27</v>
@@ -4204,16 +4286,16 @@
         <v>15</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
@@ -4225,7 +4307,7 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65" s="2" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>27</v>
@@ -4234,16 +4316,16 @@
         <v>15</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
@@ -4255,7 +4337,7 @@
     </row>
     <row r="66" spans="1:12">
       <c r="A66" s="2" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>27</v>
@@ -4264,13 +4346,13 @@
         <v>15</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
@@ -4283,7 +4365,7 @@
     </row>
     <row r="67" spans="1:12">
       <c r="A67" s="2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>27</v>
@@ -4292,16 +4374,16 @@
         <v>15</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
@@ -4313,7 +4395,7 @@
     </row>
     <row r="68" spans="1:12">
       <c r="A68" s="2" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>27</v>
@@ -4322,16 +4404,16 @@
         <v>15</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
@@ -4343,7 +4425,7 @@
     </row>
     <row r="69" spans="1:12">
       <c r="A69" s="2" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>27</v>
@@ -4352,19 +4434,19 @@
         <v>15</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="I69" s="2"/>
       <c r="J69" s="2" t="s">
@@ -4375,7 +4457,7 @@
     </row>
     <row r="70" spans="1:12">
       <c r="A70" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>27</v>
@@ -4384,19 +4466,19 @@
         <v>15</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="I70" s="2"/>
       <c r="J70" s="2" t="s">
@@ -4407,7 +4489,7 @@
     </row>
     <row r="71" spans="1:12">
       <c r="A71" s="2" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>27</v>
@@ -4416,16 +4498,16 @@
         <v>15</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>44</v>
@@ -4435,11 +4517,13 @@
         <v>4</v>
       </c>
       <c r="K71" s="8"/>
-      <c r="L71" s="2"/>
+      <c r="L71" s="2" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="72" spans="1:12">
       <c r="A72" s="2" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>27</v>
@@ -4448,13 +4532,13 @@
         <v>15</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
@@ -4467,7 +4551,7 @@
     </row>
     <row r="73" spans="1:12">
       <c r="A73" s="2" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>27</v>
@@ -4476,13 +4560,13 @@
         <v>15</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
@@ -4495,7 +4579,7 @@
     </row>
     <row r="74" spans="1:12">
       <c r="A74" s="2" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>27</v>
@@ -4504,13 +4588,13 @@
         <v>15</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
@@ -4523,7 +4607,7 @@
     </row>
     <row r="75" spans="1:12">
       <c r="A75" s="2" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>27</v>
@@ -4532,13 +4616,13 @@
         <v>15</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
@@ -4551,7 +4635,7 @@
     </row>
     <row r="76" spans="1:12">
       <c r="A76" s="2" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>27</v>
@@ -4560,13 +4644,13 @@
         <v>15</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
@@ -4579,7 +4663,7 @@
     </row>
     <row r="77" spans="1:12">
       <c r="A77" s="2" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>27</v>
@@ -4588,13 +4672,13 @@
         <v>15</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
@@ -4607,7 +4691,7 @@
     </row>
     <row r="78" spans="1:12">
       <c r="A78" s="2" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>27</v>
@@ -4616,13 +4700,13 @@
         <v>15</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
@@ -4635,7 +4719,7 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>27</v>
@@ -4644,13 +4728,13 @@
         <v>15</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
@@ -4659,11 +4743,13 @@
         <v>4</v>
       </c>
       <c r="K79" s="8"/>
-      <c r="L79" s="2"/>
+      <c r="L79" s="2" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="80" spans="1:12">
       <c r="A80" s="2" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>27</v>
@@ -4672,13 +4758,13 @@
         <v>15</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="G80" s="2"/>
       <c r="H80" s="2" t="s">
@@ -4692,12 +4778,12 @@
         <v>46278.0</v>
       </c>
       <c r="L80" s="2" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
     </row>
     <row r="81" spans="1:12">
       <c r="A81" s="2" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>27</v>
@@ -4706,13 +4792,13 @@
         <v>15</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="G81" s="2"/>
       <c r="H81" s="2" t="s">
@@ -4726,12 +4812,12 @@
         <v>46278.0</v>
       </c>
       <c r="L81" s="2" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
     </row>
     <row r="82" spans="1:12">
       <c r="A82" s="2" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>27</v>
@@ -4740,13 +4826,13 @@
         <v>15</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
@@ -4758,12 +4844,12 @@
         <v>46278.0</v>
       </c>
       <c r="L82" s="2" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
     </row>
     <row r="83" spans="1:12">
       <c r="A83" s="2" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>27</v>
@@ -4772,13 +4858,13 @@
         <v>15</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
@@ -4790,12 +4876,12 @@
         <v>46278.0</v>
       </c>
       <c r="L83" s="2" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
     </row>
     <row r="84" spans="1:12">
       <c r="A84" s="2" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>27</v>
@@ -4804,28 +4890,32 @@
         <v>15</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="G84" s="2"/>
       <c r="H84" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I84" s="2"/>
       <c r="J84" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K84" s="8"/>
-      <c r="L84" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="K84" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L84" s="2" t="s">
+        <v>284</v>
+      </c>
     </row>
     <row r="85" spans="1:12">
       <c r="A85" s="2" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>27</v>
@@ -4834,28 +4924,32 @@
         <v>15</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="G85" s="2"/>
       <c r="H85" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I85" s="2"/>
       <c r="J85" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K85" s="8"/>
-      <c r="L85" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="K85" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L85" s="2" t="s">
+        <v>287</v>
+      </c>
     </row>
     <row r="86" spans="1:12">
       <c r="A86" s="2" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>27</v>
@@ -4864,13 +4958,13 @@
         <v>15</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
@@ -4883,7 +4977,7 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87" s="2" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>27</v>
@@ -4892,13 +4986,13 @@
         <v>15</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
@@ -4911,7 +5005,7 @@
     </row>
     <row r="88" spans="1:12">
       <c r="A88" s="2" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>27</v>
@@ -4920,13 +5014,13 @@
         <v>15</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="G88" s="2"/>
       <c r="H88" s="2" t="s">
@@ -4934,14 +5028,18 @@
       </c>
       <c r="I88" s="2"/>
       <c r="J88" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K88" s="8"/>
-      <c r="L88" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="K88" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L88" s="2" t="s">
+        <v>294</v>
+      </c>
     </row>
     <row r="89" spans="1:12">
       <c r="A89" s="2" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>27</v>
@@ -4950,13 +5048,13 @@
         <v>15</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F89" s="5" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
@@ -4969,7 +5067,7 @@
     </row>
     <row r="90" spans="1:12">
       <c r="A90" s="2" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>27</v>
@@ -4978,13 +5076,13 @@
         <v>15</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F90" s="5" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
@@ -4997,7 +5095,7 @@
     </row>
     <row r="91" spans="1:12">
       <c r="A91" s="2" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>27</v>
@@ -5006,16 +5104,16 @@
         <v>15</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
@@ -5027,7 +5125,7 @@
     </row>
     <row r="92" spans="1:12">
       <c r="A92" s="2" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>27</v>
@@ -5036,13 +5134,13 @@
         <v>15</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
@@ -5055,7 +5153,7 @@
     </row>
     <row r="93" spans="1:12">
       <c r="A93" s="2" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>27</v>
@@ -5064,19 +5162,19 @@
         <v>15</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="I93" s="2"/>
       <c r="J93" s="2" t="s">
@@ -5087,7 +5185,7 @@
     </row>
     <row r="94" spans="1:12">
       <c r="A94" s="2" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>27</v>
@@ -5096,19 +5194,19 @@
         <v>15</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F94" s="5" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="I94" s="2"/>
       <c r="J94" s="2" t="s">
@@ -5119,7 +5217,7 @@
     </row>
     <row r="95" spans="1:12">
       <c r="A95" s="2" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>27</v>
@@ -5128,16 +5226,16 @@
         <v>15</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F95" s="5" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
@@ -5149,7 +5247,7 @@
     </row>
     <row r="96" spans="1:12">
       <c r="A96" s="2" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>27</v>
@@ -5158,13 +5256,13 @@
         <v>15</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F96" s="5" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
@@ -5177,7 +5275,7 @@
     </row>
     <row r="97" spans="1:12">
       <c r="A97" s="2" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>27</v>
@@ -5186,16 +5284,16 @@
         <v>15</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F97" s="5" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
@@ -5207,7 +5305,7 @@
     </row>
     <row r="98" spans="1:12">
       <c r="A98" s="2" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>27</v>
@@ -5216,16 +5314,16 @@
         <v>15</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F98" s="5" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
@@ -5237,7 +5335,7 @@
     </row>
     <row r="99" spans="1:12">
       <c r="A99" s="2" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>27</v>
@@ -5246,16 +5344,16 @@
         <v>15</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F99" s="5" t="s">
-        <v>310</v>
+        <v>323</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
@@ -5267,7 +5365,7 @@
     </row>
     <row r="100" spans="1:12">
       <c r="A100" s="2" t="s">
-        <v>311</v>
+        <v>324</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>27</v>
@@ -5276,16 +5374,16 @@
         <v>15</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
@@ -5297,7 +5395,7 @@
     </row>
     <row r="101" spans="1:12">
       <c r="A101" s="2" t="s">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>27</v>
@@ -5306,16 +5404,16 @@
         <v>15</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>314</v>
+        <v>327</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>315</v>
+        <v>328</v>
       </c>
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
@@ -5327,7 +5425,7 @@
     </row>
     <row r="102" spans="1:12">
       <c r="A102" s="2" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>27</v>
@@ -5340,7 +5438,7 @@
         <v>20</v>
       </c>
       <c r="F102" s="5" t="s">
-        <v>317</v>
+        <v>330</v>
       </c>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
@@ -5353,7 +5451,7 @@
     </row>
     <row r="103" spans="1:12">
       <c r="A103" s="2" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>27</v>
@@ -5366,10 +5464,10 @@
         <v>20</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
       <c r="H103" s="2" t="s">
         <v>39</v>
@@ -5380,12 +5478,12 @@
       </c>
       <c r="K103" s="8"/>
       <c r="L103" s="2" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
     </row>
     <row r="104" spans="1:12">
       <c r="A104" s="2" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>27</v>
@@ -5398,7 +5496,7 @@
         <v>20</v>
       </c>
       <c r="F104" s="5" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
@@ -5411,7 +5509,7 @@
     </row>
     <row r="105" spans="1:12">
       <c r="A105" s="2" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>27</v>
@@ -5424,13 +5522,13 @@
         <v>20</v>
       </c>
       <c r="F105" s="5" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="H105" s="2" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="I105" s="2"/>
       <c r="J105" s="2" t="s">
@@ -5441,7 +5539,7 @@
     </row>
     <row r="106" spans="1:12">
       <c r="A106" s="2" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>27</v>
@@ -5454,7 +5552,7 @@
         <v>21</v>
       </c>
       <c r="F106" s="5" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
@@ -5467,7 +5565,7 @@
     </row>
     <row r="107" spans="1:12">
       <c r="A107" s="2" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>27</v>
@@ -5480,7 +5578,7 @@
         <v>21</v>
       </c>
       <c r="F107" s="5" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
@@ -5493,7 +5591,7 @@
     </row>
     <row r="108" spans="1:12">
       <c r="A108" s="2" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>27</v>
@@ -5506,7 +5604,7 @@
         <v>21</v>
       </c>
       <c r="F108" s="5" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
@@ -5519,7 +5617,7 @@
     </row>
     <row r="109" spans="1:12">
       <c r="A109" s="2" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>27</v>
@@ -5532,7 +5630,7 @@
         <v>21</v>
       </c>
       <c r="F109" s="5" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
@@ -5545,7 +5643,7 @@
     </row>
     <row r="110" spans="1:12">
       <c r="A110" s="2" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>27</v>
@@ -5558,10 +5656,10 @@
         <v>23</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
@@ -5573,7 +5671,7 @@
     </row>
     <row r="111" spans="1:12">
       <c r="A111" s="2" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>27</v>
@@ -5586,10 +5684,10 @@
         <v>23</v>
       </c>
       <c r="F111" s="5" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
@@ -5601,7 +5699,7 @@
     </row>
     <row r="112" spans="1:12">
       <c r="A112" s="2" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>27</v>
@@ -5614,10 +5712,10 @@
         <v>23</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
@@ -5629,7 +5727,7 @@
     </row>
     <row r="113" spans="1:12">
       <c r="A113" s="2" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>27</v>
@@ -5642,10 +5740,10 @@
         <v>23</v>
       </c>
       <c r="F113" s="5" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="H113" s="2"/>
       <c r="I113" s="2"/>
@@ -5657,7 +5755,7 @@
     </row>
     <row r="114" spans="1:12">
       <c r="A114" s="2" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>27</v>
@@ -5670,10 +5768,10 @@
         <v>23</v>
       </c>
       <c r="F114" s="5" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="H114" s="2"/>
       <c r="I114" s="2"/>
@@ -5685,7 +5783,7 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" s="2" t="s">
-        <v>349</v>
+        <v>362</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>27</v>
@@ -5698,7 +5796,7 @@
         <v>23</v>
       </c>
       <c r="F115" s="5" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
@@ -5711,7 +5809,7 @@
     </row>
     <row r="116" spans="1:12">
       <c r="A116" s="2" t="s">
-        <v>351</v>
+        <v>364</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>27</v>
@@ -5724,7 +5822,7 @@
         <v>23</v>
       </c>
       <c r="F116" s="5" t="s">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
@@ -5737,7 +5835,7 @@
     </row>
     <row r="117" spans="1:12">
       <c r="A117" s="2" t="s">
-        <v>353</v>
+        <v>366</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>27</v>
@@ -5750,7 +5848,7 @@
         <v>23</v>
       </c>
       <c r="F117" s="5" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
@@ -5763,7 +5861,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" s="2" t="s">
-        <v>355</v>
+        <v>368</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>27</v>
@@ -5776,10 +5874,10 @@
         <v>23</v>
       </c>
       <c r="F118" s="5" t="s">
-        <v>356</v>
+        <v>369</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>357</v>
+        <v>370</v>
       </c>
       <c r="H118" s="2"/>
       <c r="I118" s="2"/>
@@ -5791,7 +5889,7 @@
     </row>
     <row r="119" spans="1:12">
       <c r="A119" s="2" t="s">
-        <v>358</v>
+        <v>371</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>27</v>
@@ -5804,10 +5902,10 @@
         <v>23</v>
       </c>
       <c r="F119" s="5" t="s">
-        <v>359</v>
+        <v>372</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>360</v>
+        <v>373</v>
       </c>
       <c r="H119" s="2"/>
       <c r="I119" s="2"/>
@@ -5819,7 +5917,7 @@
     </row>
     <row r="120" spans="1:12">
       <c r="A120" s="2" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>27</v>
@@ -5832,10 +5930,10 @@
         <v>21</v>
       </c>
       <c r="F120" s="5" t="s">
-        <v>362</v>
+        <v>375</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H120" s="2"/>
       <c r="I120" s="2"/>
@@ -5846,15 +5944,15 @@
         <v>46278.0</v>
       </c>
       <c r="L120" s="2" t="s">
-        <v>364</v>
+        <v>377</v>
       </c>
     </row>
     <row r="121" spans="1:12">
       <c r="A121" s="3" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>18</v>
@@ -5864,7 +5962,7 @@
         <v>21</v>
       </c>
       <c r="F121" s="6" t="s">
-        <v>366</v>
+        <v>379</v>
       </c>
       <c r="G121" s="3"/>
       <c r="H121" s="3"/>
@@ -5879,10 +5977,10 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" s="3" t="s">
-        <v>367</v>
+        <v>380</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>18</v>
@@ -5892,7 +5990,7 @@
         <v>21</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>368</v>
+        <v>381</v>
       </c>
       <c r="G122" s="3"/>
       <c r="H122" s="3"/>
@@ -5907,10 +6005,10 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" s="3" t="s">
-        <v>369</v>
+        <v>382</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>18</v>
@@ -5920,7 +6018,7 @@
         <v>21</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>370</v>
+        <v>383</v>
       </c>
       <c r="G123" s="3"/>
       <c r="H123" s="3"/>
@@ -5935,10 +6033,10 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" s="3" t="s">
-        <v>371</v>
+        <v>384</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C124" s="3" t="s">
         <v>18</v>
@@ -5948,7 +6046,7 @@
         <v>21</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>372</v>
+        <v>385</v>
       </c>
       <c r="G124" s="3"/>
       <c r="H124" s="3"/>
@@ -5963,10 +6061,10 @@
     </row>
     <row r="125" spans="1:12">
       <c r="A125" s="3" t="s">
-        <v>373</v>
+        <v>386</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>18</v>
@@ -5976,7 +6074,7 @@
         <v>21</v>
       </c>
       <c r="F125" s="6" t="s">
-        <v>374</v>
+        <v>387</v>
       </c>
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
@@ -5991,10 +6089,10 @@
     </row>
     <row r="126" spans="1:12">
       <c r="A126" s="3" t="s">
-        <v>375</v>
+        <v>388</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>18</v>
@@ -6004,7 +6102,7 @@
         <v>21</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
@@ -6019,10 +6117,10 @@
     </row>
     <row r="127" spans="1:12">
       <c r="A127" s="4" t="s">
-        <v>377</v>
+        <v>390</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C127" s="4" t="s">
         <v>18</v>
@@ -6032,7 +6130,7 @@
         <v>21</v>
       </c>
       <c r="F127" s="7" t="s">
-        <v>378</v>
+        <v>391</v>
       </c>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
@@ -6047,7 +6145,7 @@
     </row>
     <row r="128" spans="1:12">
       <c r="A128" s="2" t="s">
-        <v>379</v>
+        <v>392</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>27</v>
@@ -6060,14 +6158,14 @@
         <v>23</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>380</v>
+        <v>393</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>381</v>
+        <v>394</v>
       </c>
       <c r="H128" s="2"/>
       <c r="I128" s="2" t="s">
-        <v>382</v>
+        <v>395</v>
       </c>
       <c r="J128" s="2" t="s">
         <v>4</v>
@@ -6077,7 +6175,7 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" s="2" t="s">
-        <v>383</v>
+        <v>396</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>27</v>
@@ -6090,14 +6188,14 @@
         <v>23</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>384</v>
+        <v>397</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>385</v>
+        <v>398</v>
       </c>
       <c r="H129" s="2"/>
       <c r="I129" s="2" t="s">
-        <v>382</v>
+        <v>395</v>
       </c>
       <c r="J129" s="2" t="s">
         <v>4</v>
@@ -6107,10 +6205,10 @@
     </row>
     <row r="130" spans="1:12">
       <c r="A130" s="3" t="s">
-        <v>386</v>
+        <v>399</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>12</v>
@@ -6120,14 +6218,14 @@
         <v>20</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>387</v>
+        <v>400</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>388</v>
+        <v>401</v>
       </c>
       <c r="H130" s="3"/>
       <c r="I130" s="3" t="s">
-        <v>389</v>
+        <v>402</v>
       </c>
       <c r="J130" s="3" t="s">
         <v>4</v>
@@ -6137,7 +6235,7 @@
     </row>
     <row r="131" spans="1:12">
       <c r="A131" s="2" t="s">
-        <v>390</v>
+        <v>403</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>27</v>
@@ -6150,14 +6248,14 @@
         <v>22</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>391</v>
+        <v>404</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>392</v>
+        <v>405</v>
       </c>
       <c r="H131" s="2"/>
       <c r="I131" s="2" t="s">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="J131" s="2" t="s">
         <v>4</v>
@@ -6166,7 +6264,34 @@
       <c r="L131" s="2"/>
     </row>
     <row r="132" spans="1:12">
-      <c r="K132" s="11"/>
+      <c r="A132" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D132" s="2"/>
+      <c r="E132" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="H132" s="2"/>
+      <c r="I132" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J132" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K132" s="8"/>
+      <c r="L132" s="2"/>
     </row>
     <row r="133" spans="1:12">
       <c r="K133" s="11"/>

</xml_diff>

<commit_message>
ajustes de comportamiento no asociado
</commit_message>
<xml_diff>
--- a/docs/CHECKLIST_PENDIENTES.xlsx
+++ b/docs/CHECKLIST_PENDIENTES.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="430">
   <si>
     <t>NeoEduCore — Avance de pendientes</t>
   </si>
@@ -256,6 +256,9 @@
     <t>• Pregunta a responder en cada ruta: qué campos ve cada rol, no solo si llega.
 • Motivo: 5 hallazgos aparecieron por casualidad (G12, 05/08, 07/08, 08/08, 08/08 tarde) y ningún test existente los detectaba.
 • Herramienta: /security-review o /code-review sobre la rama.</t>
+  </si>
+  <si>
+    <t>Revisados los 122 endpoints contra los 4 roles. 1 hallazgo real corregido: /users era puerta paralela a /students (docente sin asignacion listaba a todos los menores con nombre y correo). Blindado por tests/Feature/Security/AlcancePorRolTest.php (13 casos). Deja abiertos S5 y S6.</t>
   </si>
   <si>
     <t>S2</t>
@@ -1284,6 +1287,69 @@
   </si>
   <si>
     <t>ESTADO_Y_PENDIENTES.md, seccion Aviso de IA e incidencias</t>
+  </si>
+  <si>
+    <t>S5</t>
+  </si>
+  <si>
+    <t>Analiticas por materia acotadas al docente</t>
+  </si>
+  <si>
+    <t>• Hoy devuelve el rendimiento de todas las materias del centro, incluidas las que no imparte.
+• Son agregados sin nombres y [173] le concede «metricas agregadas», asi que se sostiene.
+• Pero materiasDelDocente() existe y acotarlo seria coherente con el resto.</t>
+  </si>
+  <si>
+    <t>ESTADO_Y_PENDIENTES.md, Revision de alcance por rol</t>
+  </si>
+  <si>
+    <t>El docente ve solo las materias que imparte (materiasDelDocente()); el admin sigue viendolas todas. Un docente sin asignaciones recibe lista vacia.</t>
+  </si>
+  <si>
+    <t>S6</t>
+  </si>
+  <si>
+    <t>Autoria para editar y borrar calendario y recursos</t>
+  </si>
+  <si>
+    <t>• PUT/DELETE de calendar-events y study-resources no miran created_by.
+• No es fuga de datos (son escrituras y el tenant esta cerrado), pero si una puerta sobre trabajo ajeno.
+• Decision de fondo: el calendario y la biblioteca son del centro o de quien los creo?</t>
+  </si>
+  <si>
+    <t>Cada entrada es de quien la creo. El admin queda fuera de la regla (responde por la institucion). Las entradas sin autor (created_by nulo) solo las toca el admin. Regla en el trait ExigeAutoria.</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>Primaria 1-6: un solo rango de grados, y el tutor adapta el registro</t>
+  </si>
+  <si>
+    <t>• Habia tres rangos a mano que no coincidian: config 6-12, GroupController 6-12, ExamController 7-12, y los prompts decian «primaria».
+• Consecuencia real: no se podia crear un examen de 6.o aunque si el grupo.
+• Ahora los tres salen de config('academic.grade_*'), con 1-6 por defecto. Las factories tambien.
+• El tutor recibe una instruccion de registro por franja (1-2, 3-4, 5-6, y una conservadora sin grado) en las TRES superficies: chat, diagnostico y recomendaciones.</t>
+  </si>
+  <si>
+    <t>ESTADO_Y_PENDIENTES.md, Primaria 1-6</t>
+  </si>
+  <si>
+    <t>Textos de las franjas en config/openai.php (tutor.registro); logica en App\Services\AI\RegistroPorGrado.</t>
+  </si>
+  <si>
+    <t>B2a</t>
+  </si>
+  <si>
+    <t>Decidir que se hace con los datos fuera de rango</t>
+  </si>
+  <si>
+    <t>• En la base remota hay estudiantes en grados 10 y 11, grupos en 11 y examenes en 10, mas 60 estudiantes con grado NULL.
+• La validacion solo actua al escribir, asi que nada se rompe; pero esas filas ya no describen un centro de primaria.
+• Se limpian, se remapean o se dejan como datos de prueba hasta el piloto (E4)?</t>
+  </si>
+  <si>
+    <t>Lo deja abierto B2.</t>
   </si>
 </sst>
 </file>
@@ -1887,11 +1953,11 @@
       </c>
       <c r="B6">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A6,Checklist!$B$2:$B$327,"Tarea")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A6,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A6,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -1899,7 +1965,7 @@
       </c>
       <c r="E6">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A6,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F6">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A6,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
@@ -1907,11 +1973,11 @@
       </c>
       <c r="G6">
         <f>E6+F6</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H6" s="16">
         <f>IF(B6=0,0,G6/B6)</f>
-        <v>0.25</v>
+        <v>0.66666666666667</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2118,11 +2184,11 @@
       </c>
       <c r="B13">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A13,Checklist!$B$2:$B$327,"Tarea")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C13">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A13,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A13,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -2130,7 +2196,7 @@
       </c>
       <c r="E13">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A13,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13">
         <f>COUNTIFS(Checklist!$C$2:$C$327,$A13,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
@@ -2138,11 +2204,11 @@
       </c>
       <c r="G13">
         <f>E13+F13</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="16">
         <f>IF(B13=0,0,G13/B13)</f>
-        <v>0.33333333333333</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -2151,7 +2217,7 @@
       </c>
       <c r="B14" s="15">
         <f>SUM(B5:B13)</f>
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C14" s="15">
         <f>SUM(C5:C13)</f>
@@ -2163,7 +2229,7 @@
       </c>
       <c r="E14" s="15">
         <f>SUM(E5:E13)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F14" s="15">
         <f>SUM(F5:F13)</f>
@@ -2171,11 +2237,11 @@
       </c>
       <c r="G14" s="15">
         <f>SUM(G5:G13)</f>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H14" s="17">
         <f>IF(B14=0,0,G14/B14)</f>
-        <v>0.16346153846154</v>
+        <v>0.19444444444444</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -2210,11 +2276,11 @@
       </c>
       <c r="B17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -2222,7 +2288,7 @@
       </c>
       <c r="E17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F17">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A17,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
@@ -2230,11 +2296,11 @@
       </c>
       <c r="G17">
         <f>E17+F17</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H17" s="16">
         <f>IF(B17=0,0,G17/B17)</f>
-        <v>0.125</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -2243,11 +2309,11 @@
       </c>
       <c r="B18">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A18,Checklist!$B$2:$B$327,"Tarea")</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C18">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A18,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D18">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A18,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"En curso")</f>
@@ -2267,7 +2333,7 @@
       </c>
       <c r="H18" s="16">
         <f>IF(B18=0,0,G18/B18)</f>
-        <v>0.13333333333333</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2276,7 +2342,7 @@
       </c>
       <c r="B19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Pendiente")</f>
@@ -2288,7 +2354,7 @@
       </c>
       <c r="E19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Hecho")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F19">
         <f>COUNTIFS(Checklist!$E$2:$E$327,$A19,Checklist!$B$2:$B$327,"Tarea",Checklist!$J$2:$J$327,"Descartado")</f>
@@ -2296,11 +2362,11 @@
       </c>
       <c r="G19">
         <f>E19+F19</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H19" s="16">
         <f>IF(B19=0,0,G19/B19)</f>
-        <v>0.4</v>
+        <v>0.57142857142857</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -2342,7 +2408,7 @@
       </c>
       <c r="B21" s="15">
         <f>SUM(B17:B20)</f>
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C21" s="15">
         <f>SUM(C17:C20)</f>
@@ -2354,7 +2420,7 @@
       </c>
       <c r="E21" s="15">
         <f>SUM(E17:E20)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F21" s="15">
         <f>SUM(F17:F20)</f>
@@ -2362,11 +2428,11 @@
       </c>
       <c r="G21" s="15">
         <f>SUM(G17:G20)</f>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H21" s="17">
         <f>IF(B21=0,0,G21/B21)</f>
-        <v>0.16346153846154</v>
+        <v>0.19444444444444</v>
       </c>
     </row>
   </sheetData>
@@ -2750,14 +2816,18 @@
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K10" s="8"/>
-      <c r="L10" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="K10" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>27</v>
@@ -2770,10 +2840,10 @@
         <v>20</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -2785,7 +2855,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>27</v>
@@ -2798,7 +2868,7 @@
         <v>20</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -2811,10 +2881,10 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>11</v>
@@ -2824,7 +2894,7 @@
         <v>20</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -2837,10 +2907,10 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>11</v>
@@ -2850,7 +2920,7 @@
         <v>20</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
@@ -2863,7 +2933,7 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>27</v>
@@ -2876,10 +2946,10 @@
         <v>21</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -2890,12 +2960,12 @@
         <v>46278.0</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>27</v>
@@ -2908,14 +2978,14 @@
         <v>20</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>4</v>
@@ -2925,10 +2995,10 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>12</v>
@@ -2938,7 +3008,7 @@
         <v>20</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -2951,10 +3021,10 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>12</v>
@@ -2964,10 +3034,10 @@
         <v>20</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -2979,10 +3049,10 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>12</v>
@@ -2992,7 +3062,7 @@
         <v>20</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
@@ -3005,7 +3075,7 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>27</v>
@@ -3018,10 +3088,10 @@
         <v>20</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -3033,10 +3103,10 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>12</v>
@@ -3046,7 +3116,7 @@
         <v>20</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
@@ -3059,10 +3129,10 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>12</v>
@@ -3072,7 +3142,7 @@
         <v>20</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
@@ -3085,10 +3155,10 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>12</v>
@@ -3098,7 +3168,7 @@
         <v>20</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
@@ -3111,10 +3181,10 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>12</v>
@@ -3124,7 +3194,7 @@
         <v>20</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
@@ -3137,10 +3207,10 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>12</v>
@@ -3150,7 +3220,7 @@
         <v>20</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
@@ -3163,10 +3233,10 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>12</v>
@@ -3176,7 +3246,7 @@
         <v>20</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
@@ -3189,10 +3259,10 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>12</v>
@@ -3202,10 +3272,10 @@
         <v>20</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>44</v>
@@ -3219,7 +3289,7 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>27</v>
@@ -3232,10 +3302,10 @@
         <v>20</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -3247,7 +3317,7 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>27</v>
@@ -3260,14 +3330,14 @@
         <v>21</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H29" s="2"/>
       <c r="I29" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>4</v>
@@ -3277,7 +3347,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>27</v>
@@ -3290,10 +3360,10 @@
         <v>23</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
@@ -3305,7 +3375,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>27</v>
@@ -3318,10 +3388,10 @@
         <v>21</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -3333,7 +3403,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>27</v>
@@ -3346,10 +3416,10 @@
         <v>21</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -3361,7 +3431,7 @@
     </row>
     <row r="33" spans="1:12">
       <c r="A33" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>27</v>
@@ -3374,10 +3444,10 @@
         <v>23</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -3389,7 +3459,7 @@
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>27</v>
@@ -3402,13 +3472,13 @@
         <v>20</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2" t="s">
@@ -3419,7 +3489,7 @@
     </row>
     <row r="35" spans="1:12">
       <c r="A35" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>27</v>
@@ -3432,16 +3502,16 @@
         <v>23</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>4</v>
@@ -3451,7 +3521,7 @@
     </row>
     <row r="36" spans="1:12">
       <c r="A36" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>27</v>
@@ -3464,13 +3534,13 @@
         <v>23</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2" t="s">
@@ -3481,7 +3551,7 @@
     </row>
     <row r="37" spans="1:12">
       <c r="A37" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>27</v>
@@ -3494,10 +3564,10 @@
         <v>21</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -3509,7 +3579,7 @@
     </row>
     <row r="38" spans="1:12">
       <c r="A38" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>27</v>
@@ -3518,16 +3588,16 @@
         <v>14</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -3539,7 +3609,7 @@
     </row>
     <row r="39" spans="1:12">
       <c r="A39" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>27</v>
@@ -3548,16 +3618,16 @@
         <v>14</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
@@ -3569,7 +3639,7 @@
     </row>
     <row r="40" spans="1:12">
       <c r="A40" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>27</v>
@@ -3578,16 +3648,16 @@
         <v>14</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -3599,7 +3669,7 @@
     </row>
     <row r="41" spans="1:12">
       <c r="A41" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>27</v>
@@ -3608,16 +3678,16 @@
         <v>14</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
@@ -3629,7 +3699,7 @@
     </row>
     <row r="42" spans="1:12">
       <c r="A42" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>27</v>
@@ -3638,16 +3708,16 @@
         <v>14</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
@@ -3659,7 +3729,7 @@
     </row>
     <row r="43" spans="1:12">
       <c r="A43" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>27</v>
@@ -3668,16 +3738,16 @@
         <v>14</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -3689,7 +3759,7 @@
     </row>
     <row r="44" spans="1:12">
       <c r="A44" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>27</v>
@@ -3698,16 +3768,16 @@
         <v>14</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>49</v>
@@ -3718,12 +3788,12 @@
       </c>
       <c r="K44" s="8"/>
       <c r="L44" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="45" spans="1:12">
       <c r="A45" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>27</v>
@@ -3732,16 +3802,16 @@
         <v>14</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
@@ -3753,7 +3823,7 @@
     </row>
     <row r="46" spans="1:12">
       <c r="A46" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>27</v>
@@ -3762,13 +3832,13 @@
         <v>14</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
@@ -3781,7 +3851,7 @@
     </row>
     <row r="47" spans="1:12">
       <c r="A47" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>27</v>
@@ -3790,16 +3860,16 @@
         <v>14</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
@@ -3811,7 +3881,7 @@
     </row>
     <row r="48" spans="1:12">
       <c r="A48" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>27</v>
@@ -3820,16 +3890,16 @@
         <v>14</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
@@ -3841,7 +3911,7 @@
     </row>
     <row r="49" spans="1:12">
       <c r="A49" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>27</v>
@@ -3850,13 +3920,13 @@
         <v>14</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
@@ -3869,22 +3939,22 @@
     </row>
     <row r="50" spans="1:12">
       <c r="A50" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
@@ -3897,22 +3967,22 @@
     </row>
     <row r="51" spans="1:12">
       <c r="A51" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="3"/>
@@ -3925,22 +3995,22 @@
     </row>
     <row r="52" spans="1:12">
       <c r="A52" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
@@ -3953,7 +4023,7 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>27</v>
@@ -3962,16 +4032,16 @@
         <v>14</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
@@ -3983,7 +4053,7 @@
     </row>
     <row r="54" spans="1:12">
       <c r="A54" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>27</v>
@@ -3992,16 +4062,16 @@
         <v>14</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
@@ -4013,7 +4083,7 @@
     </row>
     <row r="55" spans="1:12">
       <c r="A55" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>27</v>
@@ -4022,16 +4092,16 @@
         <v>14</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
@@ -4043,7 +4113,7 @@
     </row>
     <row r="56" spans="1:12">
       <c r="A56" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>27</v>
@@ -4052,13 +4122,13 @@
         <v>14</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
@@ -4071,7 +4141,7 @@
     </row>
     <row r="57" spans="1:12">
       <c r="A57" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>27</v>
@@ -4080,16 +4150,16 @@
         <v>15</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
@@ -4101,22 +4171,22 @@
     </row>
     <row r="58" spans="1:12">
       <c r="A58" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
@@ -4129,22 +4199,22 @@
     </row>
     <row r="59" spans="1:12">
       <c r="A59" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
@@ -4157,22 +4227,22 @@
     </row>
     <row r="60" spans="1:12">
       <c r="A60" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
@@ -4185,22 +4255,22 @@
     </row>
     <row r="61" spans="1:12">
       <c r="A61" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
@@ -4213,7 +4283,7 @@
     </row>
     <row r="62" spans="1:12">
       <c r="A62" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>27</v>
@@ -4222,16 +4292,16 @@
         <v>15</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
@@ -4243,7 +4313,7 @@
     </row>
     <row r="63" spans="1:12">
       <c r="A63" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>27</v>
@@ -4252,16 +4322,16 @@
         <v>15</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>34</v>
@@ -4272,12 +4342,12 @@
       </c>
       <c r="K63" s="8"/>
       <c r="L63" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="64" spans="1:12">
       <c r="A64" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>27</v>
@@ -4286,16 +4356,16 @@
         <v>15</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
@@ -4307,7 +4377,7 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>27</v>
@@ -4316,16 +4386,16 @@
         <v>15</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
@@ -4337,7 +4407,7 @@
     </row>
     <row r="66" spans="1:12">
       <c r="A66" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>27</v>
@@ -4346,13 +4416,13 @@
         <v>15</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
@@ -4365,7 +4435,7 @@
     </row>
     <row r="67" spans="1:12">
       <c r="A67" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>27</v>
@@ -4374,16 +4444,16 @@
         <v>15</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
@@ -4395,7 +4465,7 @@
     </row>
     <row r="68" spans="1:12">
       <c r="A68" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>27</v>
@@ -4404,16 +4474,16 @@
         <v>15</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
@@ -4425,7 +4495,7 @@
     </row>
     <row r="69" spans="1:12">
       <c r="A69" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>27</v>
@@ -4434,19 +4504,19 @@
         <v>15</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I69" s="2"/>
       <c r="J69" s="2" t="s">
@@ -4457,7 +4527,7 @@
     </row>
     <row r="70" spans="1:12">
       <c r="A70" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>27</v>
@@ -4466,19 +4536,19 @@
         <v>15</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I70" s="2"/>
       <c r="J70" s="2" t="s">
@@ -4489,7 +4559,7 @@
     </row>
     <row r="71" spans="1:12">
       <c r="A71" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>27</v>
@@ -4498,16 +4568,16 @@
         <v>15</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>44</v>
@@ -4518,12 +4588,12 @@
       </c>
       <c r="K71" s="8"/>
       <c r="L71" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="72" spans="1:12">
       <c r="A72" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>27</v>
@@ -4532,13 +4602,13 @@
         <v>15</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
@@ -4551,7 +4621,7 @@
     </row>
     <row r="73" spans="1:12">
       <c r="A73" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>27</v>
@@ -4560,13 +4630,13 @@
         <v>15</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
@@ -4579,7 +4649,7 @@
     </row>
     <row r="74" spans="1:12">
       <c r="A74" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>27</v>
@@ -4588,13 +4658,13 @@
         <v>15</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
@@ -4607,7 +4677,7 @@
     </row>
     <row r="75" spans="1:12">
       <c r="A75" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>27</v>
@@ -4616,13 +4686,13 @@
         <v>15</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
@@ -4635,7 +4705,7 @@
     </row>
     <row r="76" spans="1:12">
       <c r="A76" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>27</v>
@@ -4644,13 +4714,13 @@
         <v>15</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
@@ -4663,7 +4733,7 @@
     </row>
     <row r="77" spans="1:12">
       <c r="A77" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>27</v>
@@ -4672,13 +4742,13 @@
         <v>15</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
@@ -4691,7 +4761,7 @@
     </row>
     <row r="78" spans="1:12">
       <c r="A78" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>27</v>
@@ -4700,13 +4770,13 @@
         <v>15</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
@@ -4719,7 +4789,7 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>27</v>
@@ -4728,13 +4798,13 @@
         <v>15</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
@@ -4744,12 +4814,12 @@
       </c>
       <c r="K79" s="8"/>
       <c r="L79" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="80" spans="1:12">
       <c r="A80" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>27</v>
@@ -4758,13 +4828,13 @@
         <v>15</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G80" s="2"/>
       <c r="H80" s="2" t="s">
@@ -4778,12 +4848,12 @@
         <v>46278.0</v>
       </c>
       <c r="L80" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="81" spans="1:12">
       <c r="A81" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>27</v>
@@ -4792,13 +4862,13 @@
         <v>15</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G81" s="2"/>
       <c r="H81" s="2" t="s">
@@ -4812,12 +4882,12 @@
         <v>46278.0</v>
       </c>
       <c r="L81" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="82" spans="1:12">
       <c r="A82" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>27</v>
@@ -4826,13 +4896,13 @@
         <v>15</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
@@ -4844,12 +4914,12 @@
         <v>46278.0</v>
       </c>
       <c r="L82" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="83" spans="1:12">
       <c r="A83" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>27</v>
@@ -4858,13 +4928,13 @@
         <v>15</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
@@ -4876,12 +4946,12 @@
         <v>46278.0</v>
       </c>
       <c r="L83" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="84" spans="1:12">
       <c r="A84" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>27</v>
@@ -4890,13 +4960,13 @@
         <v>15</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G84" s="2"/>
       <c r="H84" s="2" t="s">
@@ -4910,12 +4980,12 @@
         <v>46278.0</v>
       </c>
       <c r="L84" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="85" spans="1:12">
       <c r="A85" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>27</v>
@@ -4924,13 +4994,13 @@
         <v>15</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G85" s="2"/>
       <c r="H85" s="2" t="s">
@@ -4944,12 +5014,12 @@
         <v>46278.0</v>
       </c>
       <c r="L85" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="86" spans="1:12">
       <c r="A86" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>27</v>
@@ -4958,13 +5028,13 @@
         <v>15</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
@@ -4977,7 +5047,7 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>27</v>
@@ -4986,13 +5056,13 @@
         <v>15</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
@@ -5005,7 +5075,7 @@
     </row>
     <row r="88" spans="1:12">
       <c r="A88" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>27</v>
@@ -5014,13 +5084,13 @@
         <v>15</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G88" s="2"/>
       <c r="H88" s="2" t="s">
@@ -5034,12 +5104,12 @@
         <v>46278.0</v>
       </c>
       <c r="L88" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="89" spans="1:12">
       <c r="A89" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>27</v>
@@ -5048,13 +5118,13 @@
         <v>15</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F89" s="5" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
@@ -5067,7 +5137,7 @@
     </row>
     <row r="90" spans="1:12">
       <c r="A90" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>27</v>
@@ -5076,13 +5146,13 @@
         <v>15</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F90" s="5" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
@@ -5095,7 +5165,7 @@
     </row>
     <row r="91" spans="1:12">
       <c r="A91" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>27</v>
@@ -5104,16 +5174,16 @@
         <v>15</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
@@ -5125,7 +5195,7 @@
     </row>
     <row r="92" spans="1:12">
       <c r="A92" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>27</v>
@@ -5134,13 +5204,13 @@
         <v>15</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
@@ -5153,7 +5223,7 @@
     </row>
     <row r="93" spans="1:12">
       <c r="A93" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>27</v>
@@ -5162,19 +5232,19 @@
         <v>15</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I93" s="2"/>
       <c r="J93" s="2" t="s">
@@ -5185,7 +5255,7 @@
     </row>
     <row r="94" spans="1:12">
       <c r="A94" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>27</v>
@@ -5194,19 +5264,19 @@
         <v>15</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F94" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I94" s="2"/>
       <c r="J94" s="2" t="s">
@@ -5217,7 +5287,7 @@
     </row>
     <row r="95" spans="1:12">
       <c r="A95" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>27</v>
@@ -5226,16 +5296,16 @@
         <v>15</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F95" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
@@ -5247,7 +5317,7 @@
     </row>
     <row r="96" spans="1:12">
       <c r="A96" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>27</v>
@@ -5256,13 +5326,13 @@
         <v>15</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F96" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
@@ -5275,7 +5345,7 @@
     </row>
     <row r="97" spans="1:12">
       <c r="A97" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>27</v>
@@ -5284,16 +5354,16 @@
         <v>15</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F97" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
@@ -5305,7 +5375,7 @@
     </row>
     <row r="98" spans="1:12">
       <c r="A98" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>27</v>
@@ -5314,16 +5384,16 @@
         <v>15</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F98" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
@@ -5335,7 +5405,7 @@
     </row>
     <row r="99" spans="1:12">
       <c r="A99" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>27</v>
@@ -5344,16 +5414,16 @@
         <v>15</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F99" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
@@ -5365,7 +5435,7 @@
     </row>
     <row r="100" spans="1:12">
       <c r="A100" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>27</v>
@@ -5374,16 +5444,16 @@
         <v>15</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
@@ -5395,7 +5465,7 @@
     </row>
     <row r="101" spans="1:12">
       <c r="A101" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>27</v>
@@ -5404,16 +5474,16 @@
         <v>15</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
@@ -5425,7 +5495,7 @@
     </row>
     <row r="102" spans="1:12">
       <c r="A102" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>27</v>
@@ -5438,7 +5508,7 @@
         <v>20</v>
       </c>
       <c r="F102" s="5" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
@@ -5451,7 +5521,7 @@
     </row>
     <row r="103" spans="1:12">
       <c r="A103" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>27</v>
@@ -5464,10 +5534,10 @@
         <v>20</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="H103" s="2" t="s">
         <v>39</v>
@@ -5478,12 +5548,12 @@
       </c>
       <c r="K103" s="8"/>
       <c r="L103" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="104" spans="1:12">
       <c r="A104" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>27</v>
@@ -5496,7 +5566,7 @@
         <v>20</v>
       </c>
       <c r="F104" s="5" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
@@ -5509,7 +5579,7 @@
     </row>
     <row r="105" spans="1:12">
       <c r="A105" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>27</v>
@@ -5522,13 +5592,13 @@
         <v>20</v>
       </c>
       <c r="F105" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="H105" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="I105" s="2"/>
       <c r="J105" s="2" t="s">
@@ -5539,7 +5609,7 @@
     </row>
     <row r="106" spans="1:12">
       <c r="A106" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>27</v>
@@ -5552,7 +5622,7 @@
         <v>21</v>
       </c>
       <c r="F106" s="5" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
@@ -5565,7 +5635,7 @@
     </row>
     <row r="107" spans="1:12">
       <c r="A107" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>27</v>
@@ -5578,7 +5648,7 @@
         <v>21</v>
       </c>
       <c r="F107" s="5" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
@@ -5591,7 +5661,7 @@
     </row>
     <row r="108" spans="1:12">
       <c r="A108" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>27</v>
@@ -5604,7 +5674,7 @@
         <v>21</v>
       </c>
       <c r="F108" s="5" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
@@ -5617,7 +5687,7 @@
     </row>
     <row r="109" spans="1:12">
       <c r="A109" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>27</v>
@@ -5630,7 +5700,7 @@
         <v>21</v>
       </c>
       <c r="F109" s="5" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
@@ -5643,7 +5713,7 @@
     </row>
     <row r="110" spans="1:12">
       <c r="A110" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>27</v>
@@ -5656,10 +5726,10 @@
         <v>23</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
@@ -5671,7 +5741,7 @@
     </row>
     <row r="111" spans="1:12">
       <c r="A111" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>27</v>
@@ -5684,10 +5754,10 @@
         <v>23</v>
       </c>
       <c r="F111" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
@@ -5699,7 +5769,7 @@
     </row>
     <row r="112" spans="1:12">
       <c r="A112" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>27</v>
@@ -5712,10 +5782,10 @@
         <v>23</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
@@ -5727,7 +5797,7 @@
     </row>
     <row r="113" spans="1:12">
       <c r="A113" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>27</v>
@@ -5740,10 +5810,10 @@
         <v>23</v>
       </c>
       <c r="F113" s="5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="H113" s="2"/>
       <c r="I113" s="2"/>
@@ -5755,7 +5825,7 @@
     </row>
     <row r="114" spans="1:12">
       <c r="A114" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>27</v>
@@ -5768,10 +5838,10 @@
         <v>23</v>
       </c>
       <c r="F114" s="5" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="H114" s="2"/>
       <c r="I114" s="2"/>
@@ -5783,7 +5853,7 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>27</v>
@@ -5796,7 +5866,7 @@
         <v>23</v>
       </c>
       <c r="F115" s="5" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
@@ -5809,7 +5879,7 @@
     </row>
     <row r="116" spans="1:12">
       <c r="A116" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>27</v>
@@ -5822,7 +5892,7 @@
         <v>23</v>
       </c>
       <c r="F116" s="5" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
@@ -5835,7 +5905,7 @@
     </row>
     <row r="117" spans="1:12">
       <c r="A117" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>27</v>
@@ -5848,7 +5918,7 @@
         <v>23</v>
       </c>
       <c r="F117" s="5" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
@@ -5861,7 +5931,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>27</v>
@@ -5874,10 +5944,10 @@
         <v>23</v>
       </c>
       <c r="F118" s="5" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="H118" s="2"/>
       <c r="I118" s="2"/>
@@ -5889,7 +5959,7 @@
     </row>
     <row r="119" spans="1:12">
       <c r="A119" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>27</v>
@@ -5902,10 +5972,10 @@
         <v>23</v>
       </c>
       <c r="F119" s="5" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="H119" s="2"/>
       <c r="I119" s="2"/>
@@ -5917,7 +5987,7 @@
     </row>
     <row r="120" spans="1:12">
       <c r="A120" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>27</v>
@@ -5930,10 +6000,10 @@
         <v>21</v>
       </c>
       <c r="F120" s="5" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="H120" s="2"/>
       <c r="I120" s="2"/>
@@ -5944,15 +6014,15 @@
         <v>46278.0</v>
       </c>
       <c r="L120" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="121" spans="1:12">
       <c r="A121" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>18</v>
@@ -5962,7 +6032,7 @@
         <v>21</v>
       </c>
       <c r="F121" s="6" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G121" s="3"/>
       <c r="H121" s="3"/>
@@ -5977,10 +6047,10 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>18</v>
@@ -5990,7 +6060,7 @@
         <v>21</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G122" s="3"/>
       <c r="H122" s="3"/>
@@ -6005,10 +6075,10 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>18</v>
@@ -6018,7 +6088,7 @@
         <v>21</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G123" s="3"/>
       <c r="H123" s="3"/>
@@ -6033,10 +6103,10 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C124" s="3" t="s">
         <v>18</v>
@@ -6046,7 +6116,7 @@
         <v>21</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G124" s="3"/>
       <c r="H124" s="3"/>
@@ -6061,10 +6131,10 @@
     </row>
     <row r="125" spans="1:12">
       <c r="A125" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>18</v>
@@ -6074,7 +6144,7 @@
         <v>21</v>
       </c>
       <c r="F125" s="6" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
@@ -6089,10 +6159,10 @@
     </row>
     <row r="126" spans="1:12">
       <c r="A126" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>18</v>
@@ -6102,7 +6172,7 @@
         <v>21</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
@@ -6117,10 +6187,10 @@
     </row>
     <row r="127" spans="1:12">
       <c r="A127" s="4" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C127" s="4" t="s">
         <v>18</v>
@@ -6130,7 +6200,7 @@
         <v>21</v>
       </c>
       <c r="F127" s="7" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
@@ -6145,7 +6215,7 @@
     </row>
     <row r="128" spans="1:12">
       <c r="A128" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>27</v>
@@ -6158,14 +6228,14 @@
         <v>23</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H128" s="2"/>
       <c r="I128" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J128" s="2" t="s">
         <v>4</v>
@@ -6175,7 +6245,7 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>27</v>
@@ -6188,14 +6258,14 @@
         <v>23</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="H129" s="2"/>
       <c r="I129" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J129" s="2" t="s">
         <v>4</v>
@@ -6205,10 +6275,10 @@
     </row>
     <row r="130" spans="1:12">
       <c r="A130" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>12</v>
@@ -6218,14 +6288,14 @@
         <v>20</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="H130" s="3"/>
       <c r="I130" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J130" s="3" t="s">
         <v>4</v>
@@ -6235,7 +6305,7 @@
     </row>
     <row r="131" spans="1:12">
       <c r="A131" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>27</v>
@@ -6248,14 +6318,14 @@
         <v>22</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="H131" s="2"/>
       <c r="I131" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J131" s="2" t="s">
         <v>4</v>
@@ -6265,7 +6335,7 @@
     </row>
     <row r="132" spans="1:12">
       <c r="A132" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>27</v>
@@ -6278,14 +6348,14 @@
         <v>21</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="H132" s="2"/>
       <c r="I132" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J132" s="2" t="s">
         <v>4</v>
@@ -6294,16 +6364,138 @@
       <c r="L132" s="2"/>
     </row>
     <row r="133" spans="1:12">
-      <c r="K133" s="11"/>
+      <c r="A133" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D133" s="2"/>
+      <c r="E133" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="H133" s="2"/>
+      <c r="I133" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="J133" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K133" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L133" s="2" t="s">
+        <v>416</v>
+      </c>
     </row>
     <row r="134" spans="1:12">
-      <c r="K134" s="11"/>
+      <c r="A134" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D134" s="2"/>
+      <c r="E134" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="H134" s="2"/>
+      <c r="I134" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="J134" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K134" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L134" s="2" t="s">
+        <v>420</v>
+      </c>
     </row>
     <row r="135" spans="1:12">
-      <c r="K135" s="11"/>
+      <c r="A135" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D135" s="2"/>
+      <c r="E135" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="H135" s="2"/>
+      <c r="I135" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="J135" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K135" s="8">
+        <v>46278.0</v>
+      </c>
+      <c r="L135" s="2" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="136" spans="1:12">
-      <c r="K136" s="11"/>
+      <c r="A136" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D136" s="2"/>
+      <c r="E136" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="H136" s="2"/>
+      <c r="I136" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="J136" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K136" s="8"/>
+      <c r="L136" s="2" t="s">
+        <v>429</v>
+      </c>
     </row>
     <row r="137" spans="1:12">
       <c r="K137" s="11"/>

</xml_diff>

<commit_message>
ajustes de seguridad y mejoras en documentacion
</commit_message>
<xml_diff>
--- a/docs/CHECKLIST_PENDIENTES.xlsx
+++ b/docs/CHECKLIST_PENDIENTES.xlsx
@@ -4185,7 +4185,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>• (47 FK, 19 tablas de dominio = 15 entidades + 4 pivotes)</t>
+          <t>• (56 FK, 21 tablas de dominio = 17 entidades + 4 pivotes — cifras al 03/10/2026)</t>
         </is>
       </c>
       <c r="H65" s="2" t="n"/>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Añadir AiChatSession, StudentSubject y TeacherAssignment al diagrama de clases</t>
+          <t>Añadir AiChatSession, StudentSubject, TeacherAssignment y AiTutorIncident al diagrama de clases</t>
         </is>
       </c>
       <c r="G66" s="2" t="n"/>
@@ -6300,11 +6300,17 @@
       <c r="I112" s="2" t="n"/>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K112" s="8" t="n"/>
-      <c r="L112" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K112" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>Aviso en la app al activar el examen (sin correo, decisión del usuario). Frontend en F18</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6342,11 +6348,17 @@
       <c r="I113" s="2" t="n"/>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K113" s="8" t="n"/>
-      <c r="L113" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K113" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>Formato por estilo en chat y diagnóstico + campo presentation. Frontend en F19</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -6422,11 +6434,17 @@
       <c r="I115" s="2" t="n"/>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K115" s="8" t="n"/>
-      <c r="L115" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K115" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>Base temporal + migrate + dump + diff; primera ejecución sin drift. Falta CI donde engancharlo</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -6460,11 +6478,17 @@
       <c r="I116" s="2" t="n"/>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K116" s="8" t="n"/>
-      <c r="L116" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K116" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>Solo con from_group_id; la respuesta trae excluded. 3 tests en BulkReassignmentTest</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6498,11 +6522,17 @@
       <c r="I117" s="2" t="n"/>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K117" s="8" t="n"/>
-      <c r="L117" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K117" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>La petición solo encola EnviarEnlaceRecuperacion: mismo trabajo exista o no la cuenta</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6582,11 +6612,17 @@
       <c r="I119" s="2" t="n"/>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K119" s="8" t="n"/>
-      <c r="L119" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K119" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>Eran 9 modelos (también StudentSubject) + 3 FK posteriores. Vigilado por EloquentRelationsMatchFksTest</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7484,10 +7520,122 @@
       </c>
     </row>
     <row r="139">
-      <c r="K139" s="11" t="n"/>
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>F18</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>5. Frontend</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidad nueva</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>4 · Normal</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>Campanita de notificaciones</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>• GET /api/notifications (meta.unread_count), PATCH /api/notifications/{id}/read, POST /api/notifications/read-all
+• Hoy el único tipo es exam_available, con título, materia y ventana en data</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>CHECKLIST_PENDIENTES.md, sección 5</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K139" s="8" t="n"/>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>Backend listo (O1, 03/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
-      <c r="K140" s="11" t="n"/>
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>5. Frontend</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidad nueva</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>4 · Normal</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>Presentar la respuesta del tutor según presentation</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>• Con auditivo, ofrecer leerla en voz alta (p. ej. Web Speech API)
+• visual y lector llegan ya formateadas como texto</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>CHECKLIST_PENDIENTES.md, sección 5</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K140" s="8" t="n"/>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>Backend listo (O2, 03/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="K141" s="11" t="n"/>

</xml_diff>

<commit_message>
nuevo ajuste para hacer informacion que otorga el tutor sea mas orientado a lo que el tutor comparte con los estudiantes
</commit_message>
<xml_diff>
--- a/docs/CHECKLIST_PENDIENTES.xlsx
+++ b/docs/CHECKLIST_PENDIENTES.xlsx
@@ -7612,7 +7612,9 @@
       <c r="G140" s="2" t="inlineStr">
         <is>
           <t>• Con auditivo, ofrecer leerla en voz alta (p. ej. Web Speech API)
-• visual y lector llegan ya formateadas como texto</t>
+• visual y lector llegan ya formateadas como texto
+• Si viene video (visual/auditivo), incrustar el reproductor de YouTube
+• En el formulario de crear/editar examen: campo opcional video_url</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">

</xml_diff>

<commit_message>
mejoras en documentacion, comportamiento y cobertura de test
</commit_message>
<xml_diff>
--- a/docs/CHECKLIST_PENDIENTES.xlsx
+++ b/docs/CHECKLIST_PENDIENTES.xlsx
@@ -2925,11 +2925,17 @@
       <c r="I37" s="2" t="n"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K37" s="8" t="n"/>
-      <c r="L37" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Líneas 91,36 % (4271/4675) sobre 565 tests; excluye app/Console y ApiSpec (herramientas de desarrollo). Antes 77,80 %</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6396,11 +6402,17 @@
       <c r="I114" s="2" t="n"/>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K114" s="8" t="n"/>
-      <c r="L114" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K114" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>22 → 13 queries sin cola; tope de QueryBudgetTest en 14</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6570,11 +6582,17 @@
       <c r="I118" s="2" t="n"/>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K118" s="8" t="n"/>
-      <c r="L118" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K118" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>Modo opcional async:true en el chat + GET /ai/tutor/sessions/{id}. Frontend en F20</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7000,11 +7018,17 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K128" s="8" t="n"/>
-      <c r="L128" s="2" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K128" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>Decisión del usuario: se queda en UTC. La hora del centro la pinta el frontend con institutions.settings.timezone</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -7640,7 +7664,63 @@
       </c>
     </row>
     <row r="141">
-      <c r="K141" s="11" t="n"/>
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>F20</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>5. Frontend</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidad nueva</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>4 · Normal</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>Usar el chat asíncrono del tutor</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>• Mandar async:true, recibir 202 y consultar GET /api/ai/tutor/sessions/{id} hasta awaiting_reply:false
+• Con 409, esperar a la respuesta anterior</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>O7</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>CHECKLIST_PENDIENTES.md, sección 8</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K141" s="8" t="n"/>
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>Backend listo (O7, 03/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="K142" s="11" t="n"/>

</xml_diff>

<commit_message>
ajustes de comportamiento y requisitos de examen, junto con el websocket, en adicion se suman mejoras al mismo junto con mejoras en el examen
</commit_message>
<xml_diff>
--- a/docs/CHECKLIST_PENDIENTES.xlsx
+++ b/docs/CHECKLIST_PENDIENTES.xlsx
@@ -7723,25 +7723,396 @@
       </c>
     </row>
     <row r="142">
-      <c r="K142" s="11" t="n"/>
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>3. Producción y despliegue</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="n"/>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>1 · Alta</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>WebSocket (Reverb) en producción</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>• El código ya está hecho: NO es un recurso aparte; docker/entrypoint.sh arranca Reverb dentro de la App (solo con octane:start; reinicio con espera creciente; no tumba la API). Falta configurarlo en Coolify
+• Hecho: entrypoint + Dockerfile (EXPOSE 8080); probado el script con sus cuatro ramas
+• Pendiente: segundo dominio en la App hacia el puerto 8080 (https://api.…:8000,https://ws.…:8080)
+• Pendiente: variables en la App Y en el worker: BROADCAST_CONNECTION=reverb, REVERB_APP_ID, REVERB_APP_KEY, REVERB_APP_SECRET (largas y aleatorias; el secret solo en el servidor), REVERB_HOST=ws.…, REVERB_PORT=443, REVERB_SCHEME=https, REVERB_SERVER_HOST=0.0.0.0, REVERB_SERVER_PORT=8080, FRONTEND_URL
+• Pendiente: construir la imagen y comprobar en el log "[entrypoint] Arrancando Reverb…" (el daemon de Docker no estaba arrancado)
+• Pendiente: probar de punta a punta (activar un examen y verlo llegar sin recargar)
+• Una sola réplica de la App; para escalar, Redis (REVERB_SCALING_ENABLED)</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>DEPLOY_COOLIFY.md §3b</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K142" s="8" t="n"/>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>Código listo (08/10/2026); falta configuración en Coolify y prueba real.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
-      <c r="K143" s="11" t="n"/>
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>F21</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>5. Frontend</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidad nueva</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>4 · Normal</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>Aviso en vivo de examen activado (WebSocket)</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>• Laravel Echo + pusher-js con REVERB_APP_KEY, host y puerto
+• authEndpoint = /api/broadcasting/auth con el Bearer
+• Escuchar .examen.activado en el canal privado alumno.{id}
+• Payload: exam_id, title, available_from, available_until; con available_from futura, pintar «disponible desde…» y no un botón activo</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>CHECKLIST_PENDIENTES.md, sección 5</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K143" s="8" t="n"/>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>Backend listo (B4, 08/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="K144" s="11" t="n"/>
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>F22</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>5. Frontend</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidad nueva</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>4 · Normal</t>
+        </is>
+      </c>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>Enlaces de apoyo del examen</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>• Formulario de crear/editar examen: lista support_resources (hasta 5; type = video|text, url, title opcional; vídeos solo de YouTube, textos de la lista blanca)
+• Mostrar la recomendación resource con su source (teacher/catalog)
+• Mostrar el video del chat y de las recomendaciones con su title</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>CHECKLIST_PENDIENTES.md, sección 5</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K144" s="8" t="n"/>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>Backend listo (B6, 08/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
-      <c r="K145" s="11" t="n"/>
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>9. Funcionalidad nueva del backend</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="n"/>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>2 · Media</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Aviso en vivo al activar un examen (WebSocket)</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>• Laravel Reverb (proceso aparte, sin terceros). Evento ExamenActivado por la cola, canal privado por alumno (alumno.{id}) autenticado en POST /api/broadcasting/auth con el Bearer, tras el middleware activa
+• Una sola regla de quién lo ve: Exam::destinatarios(), compartida con la notificación en la app (matrícula vigente en un grupo destino, mismo centro, cuenta activa)
+• El evento informa, no autoriza: la ventana la sigue aplicando la API
+• Sin Reverb levantado no se rompe nada</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="n"/>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PENDIENTES.md, Aviso en vivo del examen activado</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K145" s="8" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>9 tests (ExamenActivadoEnVivoTest). Quedan P9 (despliegue) y F21 (frontend).</t>
+        </is>
+      </c>
     </row>
     <row r="146">
-      <c r="K146" s="11" t="n"/>
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>9. Funcionalidad nueva del backend</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="n"/>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>2 · Media</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Examen activado: evento en el calendario del aula</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>• Un evento por aula destino (Exam::publicarEnCalendario()), con las fechas de la ventana o la duración del examen, a nombre del docente
+• No duplica un evento ya puesto a mano</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="n"/>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PENDIENTES.md, Calendario</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K146" s="8" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>6 tests (ExamenEnElCalendarioTest).</t>
+        </is>
+      </c>
     </row>
     <row r="147">
-      <c r="K147" s="11" t="n"/>
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>9. Funcionalidad nueva del backend</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="n"/>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>2 · Media</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Enlaces de apoyo del examen, enlaces vivos y vídeo por edad</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>• exams.support_resources: hasta 5 enlaces de vídeo o texto que el tutor usa al recomendar; el modelo nunca elige la URL; lo del docente manda sobre la IA y sobre el catálogo
+• Antes de entregar un enlace se comprueba que responde (EnlaceDisponible): 404/410, vídeos de YouTube borrados o privados, redirecciones fuera de la lista blanca; sin veredicto = vivo; veredicto cacheado
+• Si el estilo necesita vídeo y no hay uno vivo del docente: uno del catálogo del grado del alumno (nunca de otra edad)</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="n"/>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PENDIENTES.md, Enlaces de apoyo del examen y enlaces vivos</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K147" s="8" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>25 tests (EnlacesDeApoyo… y EnlacesVivos…). Migración add_support_resources_to_exams aplicada en la base remota. Queda F22 (frontend).</t>
+        </is>
+      </c>
     </row>
     <row r="148">
-      <c r="K148" s="11" t="n"/>
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>9. Funcionalidad nueva del backend</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="n"/>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>2 · Media</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Menos tokens en el tutor</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>• Prompts recortados (3 párrafos en vez de 4) y topes más bajos: historial 20 → 10, respuesta 600 → 450, práctica 800 → 650 (.env)
+• La bajada es estimada: sin créditos de OpenAI no se pudo medir. Los textos pedagógicos quedaron más escuetos: conviene una lectura del profesorado</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="n"/>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PENDIENTES.md, Tutor IA conversacional</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="K148" s="8" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="K149" s="11" t="n"/>

</xml_diff>

<commit_message>
ajustes para separacion de instancias
</commit_message>
<xml_diff>
--- a/docs/CHECKLIST_PENDIENTES.xlsx
+++ b/docs/CHECKLIST_PENDIENTES.xlsx
@@ -7751,13 +7751,13 @@
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>• El código ya está hecho: NO es un recurso aparte; docker/entrypoint.sh arranca Reverb dentro de la App (solo con octane:start; reinicio con espera creciente; no tumba la API). Falta configurarlo en Coolify
-• Hecho: entrypoint + Dockerfile (EXPOSE 8080); probado el script con sus cuatro ramas
-• Pendiente: segundo dominio en la App hacia el puerto 8080 (https://api.…:8000,https://ws.…:8080)
-• Pendiente: variables en la App Y en el worker: BROADCAST_CONNECTION=reverb, REVERB_APP_ID, REVERB_APP_KEY, REVERB_APP_SECRET (largas y aleatorias; el secret solo en el servidor), REVERB_HOST=ws.…, REVERB_PORT=443, REVERB_SCHEME=https, REVERB_SERVER_HOST=0.0.0.0, REVERB_SERVER_PORT=8080, FRONTEND_URL
-• Pendiente: construir la imagen y comprobar en el log "[entrypoint] Arrancando Reverb…" (el daemon de Docker no estaba arrancado)
+          <t>• El código ya está hecho. Desde el 11/10/2026 son TRES instancias independientes (App, WebSocket, Worker): misma imagen, distinto comando. Falta crearlas y configurarlas en Coolify
+• Hecho: entrypoint sin Reverb embebido; docker-compose con app + websocket + queue; app y worker publican por REVERB_PUBLISH_* (red interna)
+• Pendiente: crear el recurso WebSocket (php artisan reverb:start --host=0.0.0.0 --port=8180 --no-interaction) con dominio https://ws.…:8180
+• Pendiente: variables en los TRES recursos: BROADCAST_CONNECTION=reverb, REVERB_APP_ID, REVERB_APP_KEY, REVERB_APP_SECRET (largas y aleatorias; el secret solo en el servidor), REVERB_HOST=ws.…, REVERB_PORT=443, REVERB_SCHEME=https, REVERB_SERVER_HOST=0.0.0.0, REVERB_SERVER_PORT=8180, FRONTEND_URL; más REVERB_PUBLISH_HOST/PORT/SCHEME en App y Worker
+• Pendiente: construir la imagen y probar docker compose up --build (el daemon de Docker no estaba arrancado)
 • Pendiente: probar de punta a punta (activar un examen y verlo llegar sin recargar)
-• Una sola réplica de la App; para escalar, Redis (REVERB_SCALING_ENABLED)</t>
+• Una sola réplica del WebSocket; para escalar, Redis (REVERB_SCALING_ENABLED)</t>
         </is>
       </c>
       <c r="H142" s="2" t="inlineStr">
@@ -7778,7 +7778,7 @@
       <c r="K142" s="8" t="n"/>
       <c r="L142" s="2" t="inlineStr">
         <is>
-          <t>Código listo (08/10/2026); falta configuración en Coolify y prueba real.</t>
+          <t>Código listo y separado en tres instancias (11/10/2026); falta crearlas en Coolify y prueba real.</t>
         </is>
       </c>
     </row>

</xml_diff>